<commit_message>
Add Maria Soldevila (B) solution; align (A) with professor's Exhibit 1
(A): add furniture depreciation (4,000) and website amortization (6,000),
net profit 110,000, total assets 660,000 as in Exhibit 1 of case (B).
(B): manufacturing flow (raw materials -> WIP -> finished goods),
machinery depreciation in product cost, FIFO COGS, disposal, bad debts.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012nWMFk2orvaisxGrBVUj46
</commit_message>
<xml_diff>
--- a/Accounting/Maria_Soldevila_A_solution.xlsx
+++ b/Accounting/Maria_Soldevila_A_solution.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="861" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="875" uniqueCount="493">
   <si>
     <t xml:space="preserve">FINANCIAL ACCOUNTING HOMEWORK TEMPLATE</t>
   </si>
@@ -426,16 +426,16 @@
     <t xml:space="preserve">Each sale is two entries: revenue AND cost of goods sold (Dr P&amp;L, Cr Inventories), 300 × 800.</t>
   </si>
   <si>
-    <t xml:space="preserve">Accumulated depreciation</t>
+    <t xml:space="preserve">Depreciation &amp; amortization</t>
   </si>
   <si>
     <t xml:space="preserve">empty</t>
   </si>
   <si>
-    <t xml:space="preserve">5,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The building has a 20-year life, so 100,000 / 20 = 5,000 depreciation for 2010 (Dr P&amp;L, Cr Accum. depreciation). Land is not depreciated.</t>
+    <t xml:space="preserve">15,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Building 100,000 / 20 = 5,000; furniture 20,000 / 5 = 4,000; website 12,000 / 2 = 6,000 (lives confirmed by Exhibit 1 of case B). Land is not depreciated.</t>
   </si>
   <si>
     <t xml:space="preserve">P&amp;L / Retained profits</t>
@@ -444,10 +444,10 @@
     <t xml:space="preserve">P&amp;L balance 286,000; RP empty</t>
   </si>
   <si>
-    <t xml:space="preserve">Net profit 120,000 closed to RP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Once COGS and depreciation are recorded, profit is 120,000. The closing entry moves it to retained profits.</t>
+    <t xml:space="preserve">Net profit 110,000 closed to RP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Once COGS and depreciation are recorded, profit is 110,000. The closing entry moves it to retained profits.</t>
   </si>
   <si>
     <t xml:space="preserve">Structure</t>
@@ -471,7 +471,7 @@
     <t xml:space="preserve">filled (see sheets)</t>
   </si>
   <si>
-    <t xml:space="preserve">Net profit 120,000. CFO 65,000, CFI −100,000, CFF −110,000, change in cash −145,000 (246,000 → 101,000).</t>
+    <t xml:space="preserve">Net profit 110,000. CFO 65,000, CFI −100,000, CFF −110,000, change in cash −145,000 (246,000 → 101,000).</t>
   </si>
   <si>
     <t xml:space="preserve">What you got RIGHT</t>
@@ -483,10 +483,10 @@
     <t xml:space="preserve">Assumptions made (the case gives no data)</t>
   </si>
   <si>
-    <t xml:space="preserve">• No income tax: the case gives no tax rate. If your professor uses one, tax = rate × 120,000 profit before tax.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Website (12,000) and furniture (20,000) are not amortized/depreciated because no useful life is given. Only the building is depreciated.</t>
+    <t xml:space="preserve">• No income tax: the case gives no tax rate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Furniture 5-year life and website 2-year life: not stated in case (A), taken from the professor's Exhibit 1 in case (B) (balance sheet at Dec 31, 2010).</t>
   </si>
   <si>
     <t xml:space="preserve">• Depreciation of the building is a full year (bought Dec 30, 2009).</t>
@@ -729,6 +729,21 @@
     <t xml:space="preserve">Contra-A+</t>
   </si>
   <si>
+    <t xml:space="preserve">Year-end adjustment: furniture &amp; equipment depreciation 20,000 / 5 years (per Exhibit 1 of case B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accum. depreciation – Furn. &amp; equip.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year-end adjustment: website amortization 12,000 / 2 years (per Exhibit 1 of case B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P&amp;L – Amortization expense</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accumulated amortization</t>
+  </si>
+  <si>
     <t xml:space="preserve">CE</t>
   </si>
   <si>
@@ -882,15 +897,9 @@
     <t xml:space="preserve">Mortgage / obligations on land &amp; bldgs</t>
   </si>
   <si>
-    <t xml:space="preserve">Accum. depreciation – Furn. &amp; equip.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Share premium</t>
   </si>
   <si>
-    <t xml:space="preserve">Accumulated amortization</t>
-  </si>
-  <si>
     <t xml:space="preserve">Dr: expenses</t>
   </si>
   <si>
@@ -1083,7 +1092,7 @@
     <t xml:space="preserve">By nature (Table 2): materials, personnel/salaries, depreciation, other.</t>
   </si>
   <si>
-    <t xml:space="preserve">− Depreciation expense (building 100,000 / 20)</t>
+    <t xml:space="preserve">− Depreciation &amp; amortization (building 5,000 + F&amp;E 4,000 + website 6,000)</t>
   </si>
   <si>
     <t xml:space="preserve">Homework cases often mix the two (like DSJ: salaries, rent, depreciation, other opex). That's why both kinds of line are here. Never put the same cost on two lines.</t>
@@ -1465,7 +1474,13 @@
     <t xml:space="preserve">Tips</t>
   </si>
   <si>
+    <t xml:space="preserve">F&amp;E depreciation added back</t>
+  </si>
+  <si>
     <t xml:space="preserve">If you did not record the closing entry, net profit sits in the P&amp;L row: put it in CFO there.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website amortization added back</t>
   </si>
   <si>
     <t xml:space="preserve">If you use separate accumulated depreciation accounts, the depreciation goes on those rows (CFO) and the PPE-at-cost row only shows purchases and disposals.</t>
@@ -4853,21 +4868,21 @@
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B48" s="49" t="s">
+      <c r="B48" s="49" t="n">
+        <v>12</v>
+      </c>
+      <c r="C48" s="50" t="s">
         <v>233</v>
       </c>
-      <c r="C48" s="50" t="s">
-        <v>234</v>
-      </c>
       <c r="D48" s="50" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="E48" s="51" t="n">
-        <v>120000</v>
+        <v>4000</v>
       </c>
       <c r="F48" s="51"/>
       <c r="G48" s="49" t="s">
-        <v>236</v>
+        <v>211</v>
       </c>
       <c r="H48" s="49" t="s">
         <v>230</v>
@@ -4878,19 +4893,19 @@
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B49" s="44" t="s">
-        <v>233</v>
+      <c r="B49" s="44" t="n">
+        <v>12</v>
       </c>
       <c r="C49" s="45"/>
       <c r="D49" s="45" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="E49" s="46"/>
       <c r="F49" s="46" t="n">
-        <v>120000</v>
+        <v>4000</v>
       </c>
       <c r="G49" s="44" t="s">
-        <v>171</v>
+        <v>232</v>
       </c>
       <c r="H49" s="44"/>
       <c r="I49" s="47" t="str">
@@ -4899,55 +4914,95 @@
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B50" s="49"/>
-      <c r="C50" s="50"/>
-      <c r="D50" s="50"/>
-      <c r="E50" s="51"/>
+      <c r="B50" s="49" t="n">
+        <v>13</v>
+      </c>
+      <c r="C50" s="50" t="s">
+        <v>235</v>
+      </c>
+      <c r="D50" s="50" t="s">
+        <v>236</v>
+      </c>
+      <c r="E50" s="51" t="n">
+        <v>6000</v>
+      </c>
       <c r="F50" s="51"/>
-      <c r="G50" s="49"/>
-      <c r="H50" s="49"/>
+      <c r="G50" s="49" t="s">
+        <v>211</v>
+      </c>
+      <c r="H50" s="49" t="s">
+        <v>230</v>
+      </c>
       <c r="I50" s="47" t="str">
         <f aca="false">IF(B50="","",IF(ABS(SUMIF($B$7:$B$106,B50,$E$7:$E$106)-SUMIF($B$7:$B$106,B50,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
-        <v/>
+        <v>OK</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B51" s="44"/>
+      <c r="B51" s="44" t="n">
+        <v>13</v>
+      </c>
       <c r="C51" s="45"/>
-      <c r="D51" s="45"/>
+      <c r="D51" s="45" t="s">
+        <v>237</v>
+      </c>
       <c r="E51" s="46"/>
-      <c r="F51" s="46"/>
-      <c r="G51" s="44"/>
+      <c r="F51" s="46" t="n">
+        <v>6000</v>
+      </c>
+      <c r="G51" s="44" t="s">
+        <v>232</v>
+      </c>
       <c r="H51" s="44"/>
       <c r="I51" s="47" t="str">
         <f aca="false">IF(B51="","",IF(ABS(SUMIF($B$7:$B$106,B51,$E$7:$E$106)-SUMIF($B$7:$B$106,B51,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
-        <v/>
+        <v>OK</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B52" s="49"/>
-      <c r="C52" s="50"/>
-      <c r="D52" s="50"/>
-      <c r="E52" s="51"/>
+      <c r="B52" s="49" t="s">
+        <v>238</v>
+      </c>
+      <c r="C52" s="50" t="s">
+        <v>239</v>
+      </c>
+      <c r="D52" s="50" t="s">
+        <v>240</v>
+      </c>
+      <c r="E52" s="51" t="n">
+        <v>110000</v>
+      </c>
       <c r="F52" s="51"/>
-      <c r="G52" s="49"/>
-      <c r="H52" s="49"/>
+      <c r="G52" s="49" t="s">
+        <v>241</v>
+      </c>
+      <c r="H52" s="49" t="s">
+        <v>230</v>
+      </c>
       <c r="I52" s="47" t="str">
         <f aca="false">IF(B52="","",IF(ABS(SUMIF($B$7:$B$106,B52,$E$7:$E$106)-SUMIF($B$7:$B$106,B52,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
-        <v/>
+        <v>OK</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B53" s="44"/>
+      <c r="B53" s="44" t="s">
+        <v>238</v>
+      </c>
       <c r="C53" s="45"/>
-      <c r="D53" s="45"/>
+      <c r="D53" s="45" t="s">
+        <v>242</v>
+      </c>
       <c r="E53" s="46"/>
-      <c r="F53" s="46"/>
-      <c r="G53" s="44"/>
+      <c r="F53" s="46" t="n">
+        <v>110000</v>
+      </c>
+      <c r="G53" s="44" t="s">
+        <v>171</v>
+      </c>
       <c r="H53" s="44"/>
       <c r="I53" s="47" t="str">
         <f aca="false">IF(B53="","",IF(ABS(SUMIF($B$7:$B$106,B53,$E$7:$E$106)-SUMIF($B$7:$B$106,B53,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
-        <v/>
+        <v>OK</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5718,7 +5773,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="2" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -5766,7 +5821,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="53" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C5" s="53"/>
       <c r="D5" s="53"/>
@@ -5777,7 +5832,7 @@
       <c r="I5" s="53"/>
       <c r="J5" s="53"/>
       <c r="L5" s="54" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="M5" s="54"/>
       <c r="N5" s="54"/>
@@ -5793,7 +5848,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="W6" s="48" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5816,13 +5871,13 @@
       <c r="O7" s="56"/>
       <c r="P7" s="56"/>
       <c r="R7" s="56" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="S7" s="56"/>
       <c r="T7" s="56"/>
       <c r="U7" s="56"/>
       <c r="W7" s="52" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5830,10 +5885,10 @@
         <v>107</v>
       </c>
       <c r="C8" s="58" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="D8" s="57" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="E8" s="57" t="s">
         <v>107</v>
@@ -5842,10 +5897,10 @@
         <v>107</v>
       </c>
       <c r="H8" s="58" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="I8" s="57" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="J8" s="57" t="s">
         <v>107</v>
@@ -5854,10 +5909,10 @@
         <v>107</v>
       </c>
       <c r="N8" s="58" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="O8" s="57" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="P8" s="57" t="s">
         <v>107</v>
@@ -5866,21 +5921,21 @@
         <v>107</v>
       </c>
       <c r="S8" s="58" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="T8" s="57" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="U8" s="57" t="s">
         <v>107</v>
       </c>
       <c r="W8" s="52" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="C9" s="60" t="n">
         <v>246000</v>
@@ -5888,7 +5943,7 @@
       <c r="D9" s="61"/>
       <c r="E9" s="59"/>
       <c r="G9" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="H9" s="60"/>
       <c r="I9" s="61"/>
@@ -5899,16 +5954,16 @@
         <v>12000</v>
       </c>
       <c r="P9" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="R9" s="59"/>
       <c r="S9" s="60"/>
       <c r="T9" s="61"/>
       <c r="U9" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="W9" s="52" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5949,7 +6004,7 @@
       <c r="T10" s="51"/>
       <c r="U10" s="62"/>
       <c r="W10" s="48" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5978,7 +6033,7 @@
       <c r="T11" s="51"/>
       <c r="U11" s="62"/>
       <c r="W11" s="52" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6003,7 +6058,7 @@
       <c r="T12" s="51"/>
       <c r="U12" s="62"/>
       <c r="W12" s="48" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6028,7 +6083,7 @@
       <c r="T13" s="51"/>
       <c r="U13" s="62"/>
       <c r="W13" s="52" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6053,7 +6108,7 @@
       <c r="T14" s="51"/>
       <c r="U14" s="62"/>
       <c r="W14" s="48" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6078,7 +6133,7 @@
       <c r="T15" s="51"/>
       <c r="U15" s="62"/>
       <c r="W15" s="52" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6099,7 +6154,7 @@
       <c r="T16" s="51"/>
       <c r="U16" s="62"/>
       <c r="W16" s="52" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6120,7 +6175,7 @@
       <c r="T17" s="51"/>
       <c r="U17" s="62"/>
       <c r="W17" s="48" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6141,7 +6196,7 @@
       <c r="T18" s="51"/>
       <c r="U18" s="62"/>
       <c r="W18" s="52" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6162,7 +6217,7 @@
       <c r="T19" s="51"/>
       <c r="U19" s="62"/>
       <c r="W19" s="52" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6183,7 +6238,7 @@
       <c r="T20" s="51"/>
       <c r="U20" s="62"/>
       <c r="W20" s="48" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6204,7 +6259,7 @@
       <c r="T21" s="51"/>
       <c r="U21" s="62"/>
       <c r="W21" s="52" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6225,7 +6280,7 @@
       <c r="T22" s="51"/>
       <c r="U22" s="62"/>
       <c r="W22" s="52" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6246,7 +6301,7 @@
       <c r="T23" s="51"/>
       <c r="U23" s="62"/>
       <c r="W23" s="52" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6267,12 +6322,12 @@
       <c r="T24" s="51"/>
       <c r="U24" s="62"/>
       <c r="W24" s="52" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C25" s="65" t="n">
         <f aca="false">SUM(C9:C24)</f>
@@ -6283,10 +6338,10 @@
         <v>515000</v>
       </c>
       <c r="E25" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="G25" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="H25" s="65" t="n">
         <f aca="false">SUM(H9:H24)</f>
@@ -6297,10 +6352,10 @@
         <v>0</v>
       </c>
       <c r="J25" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="M25" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="N25" s="65" t="n">
         <f aca="false">SUM(N9:N24)</f>
@@ -6311,10 +6366,10 @@
         <v>260000</v>
       </c>
       <c r="P25" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="R25" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="S25" s="65" t="n">
         <f aca="false">SUM(S9:S24)</f>
@@ -6325,15 +6380,15 @@
         <v>0</v>
       </c>
       <c r="U25" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="W25" s="52" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="67" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C26" s="68" t="n">
         <f aca="false">C25-D25</f>
@@ -6341,7 +6396,7 @@
       </c>
       <c r="D26" s="69"/>
       <c r="G26" s="67" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="H26" s="68" t="n">
         <f aca="false">H25-I25</f>
@@ -6354,7 +6409,7 @@
         <v>50000</v>
       </c>
       <c r="P26" s="72" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="S26" s="70"/>
       <c r="T26" s="71" t="n">
@@ -6362,15 +6417,15 @@
         <v>0</v>
       </c>
       <c r="U26" s="72" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="W26" s="52" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="W27" s="52" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6387,19 +6442,19 @@
       <c r="I28" s="55"/>
       <c r="J28" s="55"/>
       <c r="M28" s="56" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="N28" s="56"/>
       <c r="O28" s="56"/>
       <c r="P28" s="56"/>
       <c r="R28" s="56" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="S28" s="56"/>
       <c r="T28" s="56"/>
       <c r="U28" s="56"/>
       <c r="W28" s="52" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6407,10 +6462,10 @@
         <v>107</v>
       </c>
       <c r="C29" s="58" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="D29" s="57" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="E29" s="57" t="s">
         <v>107</v>
@@ -6419,10 +6474,10 @@
         <v>107</v>
       </c>
       <c r="H29" s="58" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="I29" s="57" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="J29" s="57" t="s">
         <v>107</v>
@@ -6431,10 +6486,10 @@
         <v>107</v>
       </c>
       <c r="N29" s="58" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="O29" s="57" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="P29" s="57" t="s">
         <v>107</v>
@@ -6443,27 +6498,27 @@
         <v>107</v>
       </c>
       <c r="S29" s="58" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="T29" s="57" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="U29" s="57" t="s">
         <v>107</v>
       </c>
       <c r="W29" s="52" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="C30" s="60"/>
       <c r="D30" s="61"/>
       <c r="E30" s="59"/>
       <c r="G30" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="H30" s="60" t="n">
         <v>24000</v>
@@ -6474,16 +6529,16 @@
       <c r="N30" s="60"/>
       <c r="O30" s="61"/>
       <c r="P30" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="R30" s="59"/>
       <c r="S30" s="60"/>
       <c r="T30" s="61"/>
       <c r="U30" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="W30" s="48" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6520,7 +6575,7 @@
       <c r="T31" s="51"/>
       <c r="U31" s="62"/>
       <c r="W31" s="52" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6781,7 +6836,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C46" s="65" t="n">
         <f aca="false">SUM(C30:C45)</f>
@@ -6792,10 +6847,10 @@
         <v>220000</v>
       </c>
       <c r="E46" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="G46" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="H46" s="65" t="n">
         <f aca="false">SUM(H30:H45)</f>
@@ -6806,10 +6861,10 @@
         <v>240000</v>
       </c>
       <c r="J46" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="M46" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="N46" s="65" t="n">
         <f aca="false">SUM(N30:N45)</f>
@@ -6820,10 +6875,10 @@
         <v>0</v>
       </c>
       <c r="P46" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="R46" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="S46" s="65" t="n">
         <f aca="false">SUM(S30:S45)</f>
@@ -6834,12 +6889,12 @@
         <v>0</v>
       </c>
       <c r="U46" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="67" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C47" s="68" t="n">
         <f aca="false">C46-D46</f>
@@ -6847,7 +6902,7 @@
       </c>
       <c r="D47" s="69"/>
       <c r="G47" s="67" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="H47" s="68" t="n">
         <f aca="false">H46-I46</f>
@@ -6860,7 +6915,7 @@
         <v>0</v>
       </c>
       <c r="P47" s="72" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="S47" s="70"/>
       <c r="T47" s="71" t="n">
@@ -6868,30 +6923,30 @@
         <v>0</v>
       </c>
       <c r="U47" s="72" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="55" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="C49" s="55"/>
       <c r="D49" s="55"/>
       <c r="E49" s="55"/>
       <c r="G49" s="55" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="H49" s="55"/>
       <c r="I49" s="55"/>
       <c r="J49" s="55"/>
       <c r="M49" s="56" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="N49" s="56"/>
       <c r="O49" s="56"/>
       <c r="P49" s="56"/>
       <c r="R49" s="56" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="S49" s="56"/>
       <c r="T49" s="56"/>
@@ -6902,10 +6957,10 @@
         <v>107</v>
       </c>
       <c r="C50" s="58" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="D50" s="57" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="E50" s="57" t="s">
         <v>107</v>
@@ -6914,10 +6969,10 @@
         <v>107</v>
       </c>
       <c r="H50" s="58" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="I50" s="57" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="J50" s="57" t="s">
         <v>107</v>
@@ -6926,10 +6981,10 @@
         <v>107</v>
       </c>
       <c r="N50" s="58" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="O50" s="57" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="P50" s="57" t="s">
         <v>107</v>
@@ -6938,10 +6993,10 @@
         <v>107</v>
       </c>
       <c r="S50" s="58" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="T50" s="57" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="U50" s="57" t="s">
         <v>107</v>
@@ -6949,13 +7004,13 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="C51" s="60"/>
       <c r="D51" s="61"/>
       <c r="E51" s="59"/>
       <c r="G51" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="H51" s="60"/>
       <c r="I51" s="61"/>
@@ -6964,13 +7019,13 @@
       <c r="N51" s="60"/>
       <c r="O51" s="61"/>
       <c r="P51" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="R51" s="59"/>
       <c r="S51" s="60"/>
       <c r="T51" s="61"/>
       <c r="U51" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7245,7 +7300,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B67" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C67" s="65" t="n">
         <f aca="false">SUM(C51:C66)</f>
@@ -7256,10 +7311,10 @@
         <v>0</v>
       </c>
       <c r="E67" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="G67" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="H67" s="65" t="n">
         <f aca="false">SUM(H51:H66)</f>
@@ -7270,10 +7325,10 @@
         <v>0</v>
       </c>
       <c r="J67" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="M67" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="N67" s="65" t="n">
         <f aca="false">SUM(N51:N66)</f>
@@ -7284,10 +7339,10 @@
         <v>0</v>
       </c>
       <c r="P67" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="R67" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="S67" s="65" t="n">
         <f aca="false">SUM(S51:S66)</f>
@@ -7298,12 +7353,12 @@
         <v>0</v>
       </c>
       <c r="U67" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B68" s="67" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C68" s="68" t="n">
         <f aca="false">C67-D67</f>
@@ -7311,7 +7366,7 @@
       </c>
       <c r="D68" s="69"/>
       <c r="G68" s="67" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="H68" s="68" t="n">
         <f aca="false">H67-I67</f>
@@ -7324,7 +7379,7 @@
         <v>0</v>
       </c>
       <c r="P68" s="72" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="S68" s="70"/>
       <c r="T68" s="71" t="n">
@@ -7332,7 +7387,7 @@
         <v>0</v>
       </c>
       <c r="U68" s="72" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7343,7 +7398,7 @@
       <c r="D70" s="55"/>
       <c r="E70" s="55"/>
       <c r="G70" s="55" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="H70" s="55"/>
       <c r="I70" s="55"/>
@@ -7366,10 +7421,10 @@
         <v>107</v>
       </c>
       <c r="C71" s="58" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="D71" s="57" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="E71" s="57" t="s">
         <v>107</v>
@@ -7378,10 +7433,10 @@
         <v>107</v>
       </c>
       <c r="H71" s="58" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="I71" s="57" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="J71" s="57" t="s">
         <v>107</v>
@@ -7390,10 +7445,10 @@
         <v>107</v>
       </c>
       <c r="N71" s="58" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="O71" s="57" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="P71" s="57" t="s">
         <v>107</v>
@@ -7402,10 +7457,10 @@
         <v>107</v>
       </c>
       <c r="S71" s="58" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="T71" s="57" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="U71" s="57" t="s">
         <v>107</v>
@@ -7413,7 +7468,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B72" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="C72" s="60" t="n">
         <v>300000</v>
@@ -7421,7 +7476,7 @@
       <c r="D72" s="61"/>
       <c r="E72" s="59"/>
       <c r="G72" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="H72" s="60"/>
       <c r="I72" s="61"/>
@@ -7432,7 +7487,7 @@
         <v>110000</v>
       </c>
       <c r="P72" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="R72" s="59"/>
       <c r="S72" s="60"/>
@@ -7440,7 +7495,7 @@
         <v>80000</v>
       </c>
       <c r="U72" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7723,7 +7778,7 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B88" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C88" s="65" t="n">
         <f aca="false">SUM(C72:C87)</f>
@@ -7734,10 +7789,10 @@
         <v>0</v>
       </c>
       <c r="E88" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="G88" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="H88" s="65" t="n">
         <f aca="false">SUM(H72:H87)</f>
@@ -7748,10 +7803,10 @@
         <v>0</v>
       </c>
       <c r="J88" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="M88" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="N88" s="65" t="n">
         <f aca="false">SUM(N72:N87)</f>
@@ -7762,10 +7817,10 @@
         <v>110000</v>
       </c>
       <c r="P88" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="R88" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="S88" s="65" t="n">
         <f aca="false">SUM(S72:S87)</f>
@@ -7776,12 +7831,12 @@
         <v>80000</v>
       </c>
       <c r="U88" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B89" s="67" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C89" s="68" t="n">
         <f aca="false">C88-D88</f>
@@ -7789,7 +7844,7 @@
       </c>
       <c r="D89" s="69"/>
       <c r="G89" s="67" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="H89" s="68" t="n">
         <f aca="false">H88-I88</f>
@@ -7802,7 +7857,7 @@
         <v>0</v>
       </c>
       <c r="P89" s="72" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="S89" s="70"/>
       <c r="T89" s="71" t="n">
@@ -7810,7 +7865,7 @@
         <v>0</v>
       </c>
       <c r="U89" s="72" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7827,13 +7882,13 @@
       <c r="I91" s="55"/>
       <c r="J91" s="55"/>
       <c r="M91" s="56" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="N91" s="56"/>
       <c r="O91" s="56"/>
       <c r="P91" s="56"/>
       <c r="R91" s="56" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="S91" s="56"/>
       <c r="T91" s="56"/>
@@ -7844,10 +7899,10 @@
         <v>107</v>
       </c>
       <c r="C92" s="58" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="D92" s="57" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="E92" s="57" t="s">
         <v>107</v>
@@ -7856,10 +7911,10 @@
         <v>107</v>
       </c>
       <c r="H92" s="58" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="I92" s="57" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="J92" s="57" t="s">
         <v>107</v>
@@ -7868,10 +7923,10 @@
         <v>107</v>
       </c>
       <c r="N92" s="58" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="O92" s="57" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="P92" s="57" t="s">
         <v>107</v>
@@ -7880,10 +7935,10 @@
         <v>107</v>
       </c>
       <c r="S92" s="58" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="T92" s="57" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="U92" s="57" t="s">
         <v>107</v>
@@ -7891,7 +7946,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B93" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="C93" s="60" t="n">
         <v>100000</v>
@@ -7902,19 +7957,19 @@
       <c r="H93" s="60"/>
       <c r="I93" s="61"/>
       <c r="J93" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="M93" s="59"/>
       <c r="N93" s="60"/>
       <c r="O93" s="61"/>
       <c r="P93" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="R93" s="59"/>
       <c r="S93" s="60"/>
       <c r="T93" s="61"/>
       <c r="U93" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8193,7 +8248,7 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B109" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C109" s="65" t="n">
         <f aca="false">SUM(C93:C108)</f>
@@ -8204,10 +8259,10 @@
         <v>0</v>
       </c>
       <c r="E109" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="G109" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="H109" s="65" t="n">
         <f aca="false">SUM(H93:H108)</f>
@@ -8218,10 +8273,10 @@
         <v>5000</v>
       </c>
       <c r="J109" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="M109" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="N109" s="65" t="n">
         <f aca="false">SUM(N93:N108)</f>
@@ -8232,10 +8287,10 @@
         <v>0</v>
       </c>
       <c r="P109" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="R109" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="S109" s="65" t="n">
         <f aca="false">SUM(S93:S108)</f>
@@ -8246,12 +8301,12 @@
         <v>0</v>
       </c>
       <c r="U109" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B110" s="67" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C110" s="68" t="n">
         <f aca="false">C109-D109</f>
@@ -8264,7 +8319,7 @@
         <v>5000</v>
       </c>
       <c r="J110" s="67" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="N110" s="70"/>
       <c r="O110" s="71" t="n">
@@ -8272,7 +8327,7 @@
         <v>0</v>
       </c>
       <c r="P110" s="72" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="S110" s="70"/>
       <c r="T110" s="71" t="n">
@@ -8280,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="U110" s="72" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8291,7 +8346,7 @@
       <c r="D112" s="55"/>
       <c r="E112" s="55"/>
       <c r="G112" s="55" t="s">
-        <v>284</v>
+        <v>234</v>
       </c>
       <c r="H112" s="55"/>
       <c r="I112" s="55"/>
@@ -8303,7 +8358,7 @@
       <c r="O112" s="74"/>
       <c r="P112" s="74"/>
       <c r="R112" s="74" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="S112" s="74"/>
       <c r="T112" s="74"/>
@@ -8314,10 +8369,10 @@
         <v>107</v>
       </c>
       <c r="C113" s="58" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="D113" s="57" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="E113" s="57" t="s">
         <v>107</v>
@@ -8326,10 +8381,10 @@
         <v>107</v>
       </c>
       <c r="H113" s="58" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="I113" s="57" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="J113" s="57" t="s">
         <v>107</v>
@@ -8338,10 +8393,10 @@
         <v>107</v>
       </c>
       <c r="N113" s="58" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="O113" s="57" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="P113" s="57" t="s">
         <v>107</v>
@@ -8350,10 +8405,10 @@
         <v>107</v>
       </c>
       <c r="S113" s="58" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="T113" s="57" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="U113" s="57" t="s">
         <v>107</v>
@@ -8361,7 +8416,7 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B114" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="C114" s="60" t="n">
         <v>20000</v>
@@ -8372,7 +8427,7 @@
       <c r="H114" s="60"/>
       <c r="I114" s="61"/>
       <c r="J114" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="M114" s="59"/>
       <c r="N114" s="60"/>
@@ -8380,13 +8435,13 @@
         <v>500000</v>
       </c>
       <c r="P114" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="R114" s="59"/>
       <c r="S114" s="60"/>
       <c r="T114" s="61"/>
       <c r="U114" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8396,8 +8451,12 @@
       <c r="E115" s="62"/>
       <c r="G115" s="62"/>
       <c r="H115" s="63"/>
-      <c r="I115" s="51"/>
-      <c r="J115" s="62"/>
+      <c r="I115" s="51" t="n">
+        <v>4000</v>
+      </c>
+      <c r="J115" s="62" t="n">
+        <v>12</v>
+      </c>
       <c r="M115" s="62"/>
       <c r="N115" s="63"/>
       <c r="O115" s="51"/>
@@ -8661,7 +8720,7 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B130" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C130" s="65" t="n">
         <f aca="false">SUM(C114:C129)</f>
@@ -8672,10 +8731,10 @@
         <v>0</v>
       </c>
       <c r="E130" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="G130" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="H130" s="65" t="n">
         <f aca="false">SUM(H114:H129)</f>
@@ -8683,13 +8742,13 @@
       </c>
       <c r="I130" s="66" t="n">
         <f aca="false">SUM(I114:I129)</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="J130" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="M130" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="N130" s="65" t="n">
         <f aca="false">SUM(N114:N129)</f>
@@ -8700,10 +8759,10 @@
         <v>500000</v>
       </c>
       <c r="P130" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="R130" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="S130" s="65" t="n">
         <f aca="false">SUM(S114:S129)</f>
@@ -8714,12 +8773,12 @@
         <v>0</v>
       </c>
       <c r="U130" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B131" s="67" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C131" s="68" t="n">
         <f aca="false">C130-D130</f>
@@ -8729,10 +8788,10 @@
       <c r="H131" s="70"/>
       <c r="I131" s="73" t="n">
         <f aca="false">I130-H130</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="J131" s="67" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="N131" s="70"/>
       <c r="O131" s="75" t="n">
@@ -8740,7 +8799,7 @@
         <v>500000</v>
       </c>
       <c r="P131" s="76" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="S131" s="70"/>
       <c r="T131" s="75" t="n">
@@ -8748,7 +8807,7 @@
         <v>0</v>
       </c>
       <c r="U131" s="76" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8759,19 +8818,19 @@
       <c r="D133" s="55"/>
       <c r="E133" s="55"/>
       <c r="G133" s="55" t="s">
-        <v>286</v>
+        <v>237</v>
       </c>
       <c r="H133" s="55"/>
       <c r="I133" s="55"/>
       <c r="J133" s="55"/>
       <c r="M133" s="74" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="N133" s="74"/>
       <c r="O133" s="74"/>
       <c r="P133" s="74"/>
       <c r="R133" s="77" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="S133" s="77"/>
       <c r="T133" s="77"/>
@@ -8782,10 +8841,10 @@
         <v>107</v>
       </c>
       <c r="C134" s="58" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="D134" s="57" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="E134" s="57" t="s">
         <v>107</v>
@@ -8794,10 +8853,10 @@
         <v>107</v>
       </c>
       <c r="H134" s="58" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="I134" s="57" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="J134" s="57" t="s">
         <v>107</v>
@@ -8806,10 +8865,10 @@
         <v>107</v>
       </c>
       <c r="N134" s="58" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="O134" s="57" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="P134" s="57" t="s">
         <v>107</v>
@@ -8818,10 +8877,10 @@
         <v>107</v>
       </c>
       <c r="S134" s="58" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="T134" s="57" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="U134" s="57" t="s">
         <v>107</v>
@@ -8829,7 +8888,7 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B135" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="C135" s="60" t="n">
         <v>12000</v>
@@ -8840,19 +8899,19 @@
       <c r="H135" s="60"/>
       <c r="I135" s="61"/>
       <c r="J135" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="M135" s="59"/>
       <c r="N135" s="60"/>
       <c r="O135" s="61"/>
       <c r="P135" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="R135" s="59"/>
       <c r="S135" s="60"/>
       <c r="T135" s="61"/>
       <c r="U135" s="59" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8862,15 +8921,19 @@
       <c r="E136" s="62"/>
       <c r="G136" s="62"/>
       <c r="H136" s="63"/>
-      <c r="I136" s="51"/>
-      <c r="J136" s="62"/>
+      <c r="I136" s="51" t="n">
+        <v>6000</v>
+      </c>
+      <c r="J136" s="62" t="n">
+        <v>13</v>
+      </c>
       <c r="M136" s="62"/>
       <c r="N136" s="63"/>
       <c r="O136" s="51" t="n">
-        <v>120000</v>
+        <v>110000</v>
       </c>
       <c r="P136" s="62" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="R136" s="62" t="s">
         <v>208</v>
@@ -8990,11 +9053,11 @@
       <c r="N141" s="63"/>
       <c r="O141" s="51"/>
       <c r="P141" s="62"/>
-      <c r="R141" s="62" t="s">
-        <v>233</v>
+      <c r="R141" s="62" t="n">
+        <v>12</v>
       </c>
       <c r="S141" s="63" t="n">
-        <v>120000</v>
+        <v>4000</v>
       </c>
       <c r="T141" s="51"/>
       <c r="U141" s="62"/>
@@ -9012,8 +9075,12 @@
       <c r="N142" s="63"/>
       <c r="O142" s="51"/>
       <c r="P142" s="62"/>
-      <c r="R142" s="62"/>
-      <c r="S142" s="63"/>
+      <c r="R142" s="62" t="n">
+        <v>13</v>
+      </c>
+      <c r="S142" s="63" t="n">
+        <v>6000</v>
+      </c>
       <c r="T142" s="51"/>
       <c r="U142" s="62"/>
     </row>
@@ -9030,8 +9097,12 @@
       <c r="N143" s="63"/>
       <c r="O143" s="51"/>
       <c r="P143" s="62"/>
-      <c r="R143" s="62"/>
-      <c r="S143" s="63"/>
+      <c r="R143" s="62" t="s">
+        <v>238</v>
+      </c>
+      <c r="S143" s="63" t="n">
+        <v>110000</v>
+      </c>
       <c r="T143" s="51"/>
       <c r="U143" s="62"/>
     </row>
@@ -9163,7 +9234,7 @@
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B151" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C151" s="65" t="n">
         <f aca="false">SUM(C135:C150)</f>
@@ -9174,10 +9245,10 @@
         <v>0</v>
       </c>
       <c r="E151" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="G151" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="H151" s="65" t="n">
         <f aca="false">SUM(H135:H150)</f>
@@ -9185,13 +9256,13 @@
       </c>
       <c r="I151" s="66" t="n">
         <f aca="false">SUM(I135:I150)</f>
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="J151" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="M151" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="N151" s="65" t="n">
         <f aca="false">SUM(N135:N150)</f>
@@ -9199,13 +9270,13 @@
       </c>
       <c r="O151" s="66" t="n">
         <f aca="false">SUM(O135:O150)</f>
-        <v>120000</v>
+        <v>110000</v>
       </c>
       <c r="P151" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="R151" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="S151" s="65" t="n">
         <f aca="false">SUM(S135:S150)</f>
@@ -9216,12 +9287,12 @@
         <v>460000</v>
       </c>
       <c r="U151" s="64" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B152" s="67" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C152" s="68" t="n">
         <f aca="false">C151-D151</f>
@@ -9231,18 +9302,18 @@
       <c r="H152" s="70"/>
       <c r="I152" s="73" t="n">
         <f aca="false">I151-H151</f>
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="J152" s="67" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="N152" s="70"/>
       <c r="O152" s="75" t="n">
         <f aca="false">O151-N151</f>
-        <v>120000</v>
+        <v>110000</v>
       </c>
       <c r="P152" s="76" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="S152" s="70"/>
       <c r="T152" s="78" t="n">
@@ -9250,12 +9321,12 @@
         <v>0</v>
       </c>
       <c r="U152" s="79" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B155" s="80" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="C155" s="80"/>
       <c r="D155" s="80"/>
@@ -9274,7 +9345,7 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B156" s="80" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="C156" s="80"/>
       <c r="D156" s="80"/>
@@ -9293,7 +9364,7 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B157" s="80" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C157" s="80"/>
       <c r="D157" s="80"/>
@@ -9388,7 +9459,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="2" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -9403,13 +9474,13 @@
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="83"/>
       <c r="C4" s="83" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="D4" s="83" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="E4" s="83" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="G4" s="43" t="s">
         <v>164</v>
@@ -9417,24 +9488,24 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="84" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C5" s="84"/>
       <c r="D5" s="84"/>
       <c r="E5" s="84"/>
       <c r="G5" s="48" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="85" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C6" s="86"/>
       <c r="D6" s="86"/>
       <c r="E6" s="86"/>
       <c r="G6" s="52" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9455,7 +9526,7 @@
         <v>-145000</v>
       </c>
       <c r="G7" s="52" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9476,7 +9547,7 @@
         <v>20000</v>
       </c>
       <c r="G8" s="48" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9497,7 +9568,7 @@
         <v>90000</v>
       </c>
       <c r="G9" s="52" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9518,7 +9589,7 @@
         <v>8000</v>
       </c>
       <c r="G10" s="52" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9539,7 +9610,7 @@
         <v>0</v>
       </c>
       <c r="G11" s="52" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9560,12 +9631,12 @@
         <v>0</v>
       </c>
       <c r="G12" s="52" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="85" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="C13" s="89" t="n">
         <f aca="false">C7+C8+C9+C10+C11+C12</f>
@@ -9580,18 +9651,18 @@
         <v>-27000</v>
       </c>
       <c r="G13" s="52" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="85" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="C14" s="86"/>
       <c r="D14" s="86"/>
       <c r="E14" s="86"/>
       <c r="G14" s="48" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9612,7 +9683,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="52" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9633,7 +9704,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="48" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9654,12 +9725,12 @@
         <v>-5000</v>
       </c>
       <c r="G17" s="52" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="22" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="C18" s="90" t="n">
         <f aca="false">C16+C17</f>
@@ -9674,7 +9745,7 @@
         <v>-5000</v>
       </c>
       <c r="G18" s="48" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9695,7 +9766,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="52" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9709,16 +9780,16 @@
       </c>
       <c r="D20" s="87" t="n">
         <f aca="false">-'T-Accounts'!$I$131</f>
-        <v>-0</v>
+        <v>-4000</v>
       </c>
       <c r="E20" s="88" t="n">
         <f aca="false">D20-C20</f>
-        <v>0</v>
+        <v>-4000</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="22" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="C21" s="90" t="n">
         <f aca="false">C19+C20</f>
@@ -9726,11 +9797,11 @@
       </c>
       <c r="D21" s="90" t="n">
         <f aca="false">D19+D20</f>
-        <v>20000</v>
+        <v>16000</v>
       </c>
       <c r="E21" s="90" t="n">
         <f aca="false">E19+E20</f>
-        <v>0</v>
+        <v>-4000</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9762,16 +9833,16 @@
       </c>
       <c r="D23" s="87" t="n">
         <f aca="false">-'T-Accounts'!$I$152</f>
-        <v>-0</v>
+        <v>-6000</v>
       </c>
       <c r="E23" s="88" t="n">
         <f aca="false">D23-C23</f>
-        <v>0</v>
+        <v>-6000</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="22" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C24" s="90" t="n">
         <f aca="false">C22+C23</f>
@@ -9779,11 +9850,11 @@
       </c>
       <c r="D24" s="90" t="n">
         <f aca="false">D22+D23</f>
-        <v>12000</v>
+        <v>6000</v>
       </c>
       <c r="E24" s="90" t="n">
         <f aca="false">E22+E23</f>
-        <v>0</v>
+        <v>-6000</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9806,7 +9877,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="85" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C26" s="89" t="n">
         <f aca="false">C15+C18+C21+C24+C25</f>
@@ -9814,16 +9885,16 @@
       </c>
       <c r="D26" s="89" t="n">
         <f aca="false">D15+D18+D21+D24+D25</f>
-        <v>427000</v>
+        <v>417000</v>
       </c>
       <c r="E26" s="89" t="n">
         <f aca="false">E15+E18+E21+E24+E25</f>
-        <v>-5000</v>
+        <v>-15000</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="91" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="C27" s="92" t="n">
         <f aca="false">C13+C26</f>
@@ -9831,16 +9902,16 @@
       </c>
       <c r="D27" s="92" t="n">
         <f aca="false">D13+D26</f>
-        <v>670000</v>
+        <v>660000</v>
       </c>
       <c r="E27" s="92" t="n">
         <f aca="false">E13+E26</f>
-        <v>-32000</v>
+        <v>-42000</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="93" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="C29" s="93"/>
       <c r="D29" s="93"/>
@@ -9901,11 +9972,11 @@
       </c>
       <c r="D33" s="87" t="n">
         <f aca="false">'T-Accounts'!$O$152</f>
-        <v>120000</v>
+        <v>110000</v>
       </c>
       <c r="E33" s="88" t="n">
         <f aca="false">D33-C33</f>
-        <v>120000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9928,7 +9999,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="94" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="C35" s="96" t="n">
         <f aca="false">C31+C32+C33+C34</f>
@@ -9936,16 +10007,16 @@
       </c>
       <c r="D35" s="96" t="n">
         <f aca="false">D31+D32+D33+D34</f>
-        <v>620000</v>
+        <v>610000</v>
       </c>
       <c r="E35" s="96" t="n">
         <f aca="false">E31+E32+E33+E34</f>
-        <v>120000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="97" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="C36" s="98"/>
       <c r="D36" s="98"/>
@@ -9989,7 +10060,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="97" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="C39" s="99" t="n">
         <f aca="false">C37+C38</f>
@@ -10006,7 +10077,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="97" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="C40" s="98"/>
       <c r="D40" s="98"/>
@@ -10158,7 +10229,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="97" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C49" s="99" t="n">
         <f aca="false">C41+C42+C43+C44+C45+C46+C47+C48</f>
@@ -10175,7 +10246,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="97" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="C50" s="99" t="n">
         <f aca="false">C39+C49</f>
@@ -10192,7 +10263,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="100" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C51" s="101" t="n">
         <f aca="false">C35+C50</f>
@@ -10200,16 +10271,16 @@
       </c>
       <c r="D51" s="101" t="n">
         <f aca="false">D35+D50</f>
-        <v>670000</v>
+        <v>660000</v>
       </c>
       <c r="E51" s="101" t="n">
         <f aca="false">E35+E50</f>
-        <v>-32000</v>
+        <v>-42000</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B53" s="28" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="C53" s="10" t="str">
         <f aca="false">IF(ABS(C27-C51)&lt;0.5,"OK","ERROR: "&amp;TEXT(C27-C51,"#,##0"))</f>
@@ -10222,7 +10293,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B54" s="28" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="D54" s="10" t="str">
         <f aca="false">'T-Accounts'!$L$157</f>
@@ -10231,7 +10302,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B56" s="28" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="C56" s="102"/>
       <c r="D56" s="102"/>
@@ -10239,7 +10310,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B57" s="22" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="C57" s="87" t="n">
         <f aca="false">C13-C49</f>
@@ -10252,7 +10323,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="22" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="C58" s="87" t="n">
         <f aca="false">C27-C50</f>
@@ -10260,12 +10331,12 @@
       </c>
       <c r="D58" s="87" t="n">
         <f aca="false">D27-D50</f>
-        <v>620000</v>
+        <v>610000</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B59" s="22" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="C59" s="103" t="n">
         <f aca="false">IF(C35=0,"-",C50/C35)</f>
@@ -10273,12 +10344,12 @@
       </c>
       <c r="D59" s="103" t="n">
         <f aca="false">IF(D35=0,"-",D50/D35)</f>
-        <v>0.0806451612903226</v>
+        <v>0.0819672131147541</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B60" s="22" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="C60" s="103" t="n">
         <f aca="false">IF(C49=0,"-",C13/C49)</f>
@@ -10340,7 +10411,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="104" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="C1" s="104"/>
       <c r="D1" s="104"/>
@@ -10353,10 +10424,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C4" s="83" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="D4" s="83" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="F4" s="43" t="s">
         <v>164</v>
@@ -10364,7 +10435,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="22" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="C5" s="51" t="n">
         <v>460000</v>
@@ -10374,12 +10445,12 @@
         <v>1</v>
       </c>
       <c r="F5" s="48" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="22" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="C6" s="51" t="n">
         <v>-240000</v>
@@ -10389,12 +10460,12 @@
         <v>-0.521739130434783</v>
       </c>
       <c r="F6" s="52" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="106" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="C7" s="107" t="n">
         <f aca="false">C5+C6</f>
@@ -10405,12 +10476,12 @@
         <v>0.478260869565217</v>
       </c>
       <c r="F7" s="48" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="22" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="C8" s="51" t="n">
         <v>-90000</v>
@@ -10420,12 +10491,12 @@
         <v>-0.195652173913044</v>
       </c>
       <c r="F8" s="52" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="22" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="C9" s="51"/>
       <c r="D9" s="105" t="str">
@@ -10433,12 +10504,12 @@
         <v/>
       </c>
       <c r="F9" s="52" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="22" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="C10" s="51"/>
       <c r="D10" s="105" t="str">
@@ -10446,12 +10517,12 @@
         <v/>
       </c>
       <c r="F10" s="48" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="22" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="C11" s="51"/>
       <c r="D11" s="105" t="str">
@@ -10459,12 +10530,12 @@
         <v/>
       </c>
       <c r="F11" s="52" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="22" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="C12" s="51"/>
       <c r="D12" s="105" t="str">
@@ -10472,27 +10543,27 @@
         <v/>
       </c>
       <c r="F12" s="52" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="22" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="C13" s="51" t="n">
-        <v>-5000</v>
+        <v>-15000</v>
       </c>
       <c r="D13" s="105" t="n">
         <f aca="false">IF(OR($C$5=0,C13=""),"",C13/$C$5)</f>
-        <v>-0.0108695652173913</v>
+        <v>-0.0326086956521739</v>
       </c>
       <c r="F13" s="52" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="22" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="C14" s="51"/>
       <c r="D14" s="105" t="str">
@@ -10500,12 +10571,12 @@
         <v/>
       </c>
       <c r="F14" s="48" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="22" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="C15" s="51"/>
       <c r="D15" s="105" t="str">
@@ -10513,28 +10584,28 @@
         <v/>
       </c>
       <c r="F15" s="52" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="106" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="C16" s="107" t="n">
         <f aca="false">C7+C8+C9+C10+C11+C12+C13+C14+C15</f>
-        <v>125000</v>
+        <v>115000</v>
       </c>
       <c r="D16" s="108" t="n">
         <f aca="false">IF(OR($C$5=0,C16=""),"",C16/$C$5)</f>
-        <v>0.271739130434783</v>
+        <v>0.25</v>
       </c>
       <c r="F16" s="52" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="22" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="C17" s="51"/>
       <c r="D17" s="105" t="str">
@@ -10542,12 +10613,12 @@
         <v/>
       </c>
       <c r="F17" s="52" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="22" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="C18" s="51" t="n">
         <v>-5000</v>
@@ -10557,28 +10628,28 @@
         <v>-0.0108695652173913</v>
       </c>
       <c r="F18" s="52" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="106" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="C19" s="107" t="n">
         <f aca="false">C16+C17+C18</f>
-        <v>120000</v>
+        <v>110000</v>
       </c>
       <c r="D19" s="108" t="n">
         <f aca="false">IF(OR($C$5=0,C19=""),"",C19/$C$5)</f>
-        <v>0.260869565217391</v>
+        <v>0.239130434782609</v>
       </c>
       <c r="F19" s="52" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="22" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="C20" s="51" t="n">
         <v>0</v>
@@ -10588,28 +10659,28 @@
         <v>0</v>
       </c>
       <c r="F20" s="52" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="106" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="C21" s="107" t="n">
         <f aca="false">C19+C20</f>
-        <v>120000</v>
+        <v>110000</v>
       </c>
       <c r="D21" s="108" t="n">
         <f aca="false">IF(OR($C$5=0,C21=""),"",C21/$C$5)</f>
-        <v>0.260869565217391</v>
+        <v>0.239130434782609</v>
       </c>
       <c r="F21" s="52" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="22" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="C22" s="51"/>
       <c r="D22" s="105" t="str">
@@ -10617,28 +10688,28 @@
         <v/>
       </c>
       <c r="F22" s="48" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="109" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="C23" s="110" t="n">
         <f aca="false">C21+C22</f>
-        <v>120000</v>
+        <v>110000</v>
       </c>
       <c r="D23" s="111" t="n">
         <f aca="false">IF(OR($C$5=0,C23=""),"",C23/$C$5)</f>
-        <v>0.260869565217391</v>
+        <v>0.239130434782609</v>
       </c>
       <c r="F23" s="52" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="22" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="C24" s="51"/>
       <c r="D24" s="105" t="str">
@@ -10646,64 +10717,64 @@
         <v/>
       </c>
       <c r="F24" s="52" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="106" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="C25" s="107" t="n">
         <f aca="false">C23+C24</f>
-        <v>120000</v>
+        <v>110000</v>
       </c>
       <c r="D25" s="108" t="n">
         <f aca="false">IF(OR($C$5=0,C25=""),"",C25/$C$5)</f>
-        <v>0.260869565217391</v>
+        <v>0.239130434782609</v>
       </c>
       <c r="F25" s="48" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F26" s="52" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="28" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="C27" s="102"/>
       <c r="D27" s="102"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="22" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="C28" s="87" t="n">
         <f aca="false">-C13</f>
-        <v>5000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="22" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="C29" s="51"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="28" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="C31" s="40" t="n">
         <f aca="false">(SUM('T-Accounts'!$T$135:$T$150)-SUMIF('T-Accounts'!$U$135:$U$150,"CE",'T-Accounts'!$T$135:$T$150))-(SUM('T-Accounts'!$S$135:$S$150)-SUMIF('T-Accounts'!$R$135:$R$150,"CE",'T-Accounts'!$S$135:$S$150))</f>
-        <v>120000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="28" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="C32" s="10" t="str">
         <f aca="false">IF(ABS(C23-C31)&lt;0.5,"OK","ERROR: "&amp;TEXT(C23-C31,"#,##0"))</f>
@@ -10751,7 +10822,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="112" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="C1" s="112"/>
     </row>
@@ -10763,7 +10834,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="113" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="C4" s="113"/>
       <c r="F4" s="43" t="s">
@@ -10772,215 +10843,215 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="25" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="C5" s="114"/>
       <c r="F5" s="48" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="22" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="C6" s="51" t="n">
         <v>370000</v>
       </c>
       <c r="F6" s="52" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="22" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="C7" s="51"/>
       <c r="F7" s="48" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="22" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="C8" s="51" t="n">
         <v>-210000</v>
       </c>
       <c r="F8" s="52" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="22" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="C9" s="51"/>
       <c r="F9" s="52" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="22" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="C10" s="51"/>
       <c r="F10" s="48" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="22" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="C11" s="51" t="n">
         <v>-90000</v>
       </c>
       <c r="F11" s="52" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="22" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="C12" s="51" t="n">
         <v>-5000</v>
       </c>
       <c r="F12" s="52" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="22" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="C13" s="51"/>
       <c r="F13" s="52" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="25" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="C14" s="115" t="n">
         <f aca="false">C6+C7+C8+C9+C10+C11+C12+C13</f>
         <v>65000</v>
       </c>
       <c r="F14" s="52" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F15" s="52" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="26" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="C16" s="116"/>
       <c r="F16" s="52" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="22" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="C17" s="51"/>
       <c r="F17" s="52" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="22" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="C18" s="51" t="n">
         <v>-80000</v>
       </c>
       <c r="F18" s="48" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="22" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="C19" s="51"/>
       <c r="F19" s="52" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="22" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="C20" s="51" t="n">
         <v>-20000</v>
       </c>
       <c r="F20" s="52" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="22" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="C21" s="51"/>
       <c r="F21" s="52" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="22" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="C22" s="51"/>
       <c r="F22" s="48" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="26" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="C23" s="117" t="n">
         <f aca="false">C17+C18+C19+C20+C21+C22</f>
         <v>-100000</v>
       </c>
       <c r="F23" s="52" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F24" s="52" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="27" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="C25" s="118"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="22" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="C26" s="51"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="22" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="C27" s="51"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="22" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="C28" s="51" t="n">
         <v>-110000</v>
@@ -10988,13 +11059,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="22" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="C29" s="51"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="27" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="C30" s="119" t="n">
         <f aca="false">C26+C27+C28+C29</f>
@@ -11003,7 +11074,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="120" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="C32" s="121" t="n">
         <f aca="false">C14+C23+C30</f>
@@ -11012,7 +11083,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="22" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="C33" s="87" t="n">
         <f aca="false">'Balance Sheet'!C7</f>
@@ -11021,7 +11092,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="22" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="C34" s="87" t="n">
         <f aca="false">C32</f>
@@ -11030,7 +11101,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="3" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="C35" s="122" t="n">
         <f aca="false">C33+C32</f>
@@ -11039,7 +11110,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="28" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="C36" s="10" t="str">
         <f aca="false">IF(ABS(C35-'Balance Sheet'!D7)&lt;0.5,"OK","ERROR: "&amp;TEXT(C35-'Balance Sheet'!D7,"#,##0"))</f>
@@ -11048,7 +11119,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="22" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="C37" s="87" t="n">
         <f aca="false">C14+C23</f>
@@ -11057,37 +11128,37 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="113" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="C39" s="113"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="25" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="C40" s="114"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="22" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="C41" s="87" t="n">
         <f aca="false">'Income Statement'!C23</f>
-        <v>120000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="22" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="C42" s="87" t="n">
         <f aca="false">'Income Statement'!C28</f>
-        <v>5000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="22" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="C43" s="87" t="n">
         <f aca="false">-'Income Statement'!C29</f>
@@ -11096,7 +11167,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="22" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="C44" s="87" t="n">
         <f aca="false">-'Balance Sheet'!E9</f>
@@ -11105,7 +11176,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="22" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="C45" s="87" t="n">
         <f aca="false">-'Balance Sheet'!E10</f>
@@ -11114,7 +11185,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="22" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="C46" s="87" t="n">
         <f aca="false">-'Balance Sheet'!E11</f>
@@ -11123,7 +11194,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="22" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="C47" s="87" t="n">
         <f aca="false">-'Balance Sheet'!E12</f>
@@ -11132,7 +11203,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="22" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="C48" s="87" t="n">
         <f aca="false">'Balance Sheet'!E41</f>
@@ -11141,7 +11212,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="22" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="C49" s="87" t="n">
         <f aca="false">'Balance Sheet'!E42</f>
@@ -11150,7 +11221,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="22" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="C50" s="87" t="n">
         <f aca="false">'Balance Sheet'!E43</f>
@@ -11159,7 +11230,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="22" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="C51" s="87" t="n">
         <f aca="false">'Balance Sheet'!E44</f>
@@ -11168,7 +11239,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="22" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="C52" s="87" t="n">
         <f aca="false">'Balance Sheet'!E45</f>
@@ -11177,7 +11248,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B53" s="25" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C53" s="115" t="n">
         <f aca="false">C41+C42+C43+C44+C45+C46+C47+C48+C49+C50+C51+C52</f>
@@ -11186,7 +11257,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B54" s="28" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="C54" s="10" t="str">
         <f aca="false">IF(ABS(C53-C14)&lt;0.5,"OK","ERROR: "&amp;TEXT(C53-C14,"#,##0"))</f>
@@ -11195,7 +11266,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B55" s="28" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="C55" s="10" t="str">
         <f aca="false">IF(ABS(C53+C23+C30-'Balance Sheet'!E7)&lt;0.5,"OK","ERROR: "&amp;TEXT(C53+C23+C30-'Balance Sheet'!E7,"#,##0"))</f>
@@ -11263,7 +11334,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="123" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="C1" s="123"/>
       <c r="D1" s="123"/>
@@ -11280,25 +11351,25 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="124" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="C4" s="124" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="D4" s="125" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="E4" s="126" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="F4" s="127" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="G4" s="124" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="H4" s="124" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="J4" s="43" t="s">
         <v>164</v>
@@ -11306,7 +11377,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="128" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="C5" s="128"/>
       <c r="D5" s="128"/>
@@ -11315,7 +11386,7 @@
       <c r="G5" s="128"/>
       <c r="H5" s="128"/>
       <c r="J5" s="48" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11337,10 +11408,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="129" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="J6" s="52" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11362,10 +11433,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="129" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="J7" s="52" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11387,10 +11458,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="129" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="J8" s="48" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11411,7 +11482,7 @@
       </c>
       <c r="H9" s="129"/>
       <c r="J9" s="52" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11432,7 +11503,7 @@
       </c>
       <c r="H10" s="129"/>
       <c r="J10" s="52" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11453,7 +11524,7 @@
       </c>
       <c r="H11" s="129"/>
       <c r="J11" s="52" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11474,7 +11545,7 @@
       </c>
       <c r="H12" s="129"/>
       <c r="J12" s="52" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11495,7 +11566,7 @@
       </c>
       <c r="H13" s="129"/>
       <c r="J13" s="48" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11516,7 +11587,7 @@
       </c>
       <c r="H14" s="129"/>
       <c r="J14" s="52" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11537,12 +11608,12 @@
       </c>
       <c r="H15" s="129"/>
       <c r="J15" s="52" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="128" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="C16" s="128"/>
       <c r="D16" s="128"/>
@@ -11551,7 +11622,7 @@
       <c r="G16" s="128"/>
       <c r="H16" s="128"/>
       <c r="J16" s="52" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11573,10 +11644,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="129" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="J17" s="48" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11586,18 +11657,22 @@
       </c>
       <c r="C18" s="87" t="n">
         <f aca="false">-'Balance Sheet'!E20</f>
-        <v>-0</v>
-      </c>
-      <c r="D18" s="51"/>
+        <v>4000</v>
+      </c>
+      <c r="D18" s="51" t="n">
+        <v>4000</v>
+      </c>
       <c r="E18" s="51"/>
       <c r="F18" s="51"/>
       <c r="G18" s="87" t="n">
         <f aca="false">C18-SUM(D18:F18)</f>
-        <v>-0</v>
-      </c>
-      <c r="H18" s="129"/>
+        <v>0</v>
+      </c>
+      <c r="H18" s="129" t="s">
+        <v>480</v>
+      </c>
       <c r="J18" s="52" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11607,18 +11682,22 @@
       </c>
       <c r="C19" s="87" t="n">
         <f aca="false">-'Balance Sheet'!E23</f>
-        <v>-0</v>
-      </c>
-      <c r="D19" s="51"/>
+        <v>6000</v>
+      </c>
+      <c r="D19" s="51" t="n">
+        <v>6000</v>
+      </c>
       <c r="E19" s="51"/>
       <c r="F19" s="51"/>
       <c r="G19" s="87" t="n">
         <f aca="false">C19-SUM(D19:F19)</f>
-        <v>-0</v>
-      </c>
-      <c r="H19" s="129"/>
+        <v>0</v>
+      </c>
+      <c r="H19" s="129" t="s">
+        <v>482</v>
+      </c>
       <c r="J19" s="52" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11651,7 +11730,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="129" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11763,7 +11842,7 @@
         <v>0</v>
       </c>
       <c r="H27" s="129" t="s">
-        <v>480</v>
+        <v>485</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11785,7 +11864,7 @@
         <v>0</v>
       </c>
       <c r="H28" s="129" t="s">
-        <v>481</v>
+        <v>486</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11878,10 +11957,10 @@
       </c>
       <c r="C34" s="87" t="n">
         <f aca="false">'Balance Sheet'!E33</f>
-        <v>120000</v>
+        <v>110000</v>
       </c>
       <c r="D34" s="51" t="n">
-        <v>120000</v>
+        <v>110000</v>
       </c>
       <c r="E34" s="51"/>
       <c r="F34" s="51"/>
@@ -11890,7 +11969,7 @@
         <v>0</v>
       </c>
       <c r="H34" s="129" t="s">
-        <v>482</v>
+        <v>487</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11913,7 +11992,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="120" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
       <c r="C36" s="132" t="n">
         <f aca="false">SUM(C6:C35)</f>
@@ -11939,7 +12018,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="28" t="s">
-        <v>484</v>
+        <v>489</v>
       </c>
       <c r="C38" s="10" t="str">
         <f aca="false">IF(ABS(C36-'Balance Sheet'!E7)&lt;0.5,"OK","ERROR: "&amp;TEXT(C36-'Balance Sheet'!E7,"#,##0"))</f>
@@ -11948,7 +12027,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="28" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="C39" s="10" t="str">
         <f aca="false">IF(SUMPRODUCT(ABS(G6:G35))&lt;0.5,"OK","ERROR: "&amp;TEXT(SUMPRODUCT(ABS(G6:G35)),"#,##0"))</f>
@@ -11957,7 +12036,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="28" t="s">
-        <v>486</v>
+        <v>491</v>
       </c>
       <c r="C40" s="10" t="str">
         <f aca="false">IF(ABS(ABS(D36-'Cash Flow'!C14)+ABS(E36-'Cash Flow'!C23)+ABS(F36-'Cash Flow'!C30))&lt;0.5,"OK","ERROR: "&amp;TEXT(ABS(D36-'Cash Flow'!C14)+ABS(E36-'Cash Flow'!C23)+ABS(F36-'Cash Flow'!C30),"#,##0"))</f>
@@ -12088,7 +12167,7 @@
         <v>Other current asset (rename)</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12124,7 +12203,7 @@
         <v>Accum. depreciation – Buildings</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>